<commit_message>
Simplify CJM workbook intake
</commit_message>
<xml_diff>
--- a/backend/data/templates/cjm_mvp_collection_template.xlsx
+++ b/backend/data/templates/cjm_mvp_collection_template.xlsx
@@ -11,25 +11,23 @@
     <sheet name="01_Паспорт проекта" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="02_ЛПР" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03_Важности ЛПР" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04_История опросов" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05_Барьеры" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06_Ожидания клиента" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07_KPI" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="08_Каналы взаимодействия" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09_Планы устранения" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10_Что нужно дозапросить" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="04_Барьеры" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05_Ожидания клиента" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_KPI и критерии успеха" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_Каналы взаимодействия" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_Планы действий" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09_Что нужно дозапросить" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Паспорт проекта'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_ЛПР'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Паспорт проекта'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_ЛПР'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Важности ЛПР'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_История опросов'!$A$1:$N$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Барьеры'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_Ожидания клиента'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_KPI'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_Каналы взаимодействия'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_Планы устранения'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_Что нужно дозапросить'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Барьеры'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Ожидания клиента'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_KPI и критерии успеха'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_Каналы взаимодействия'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_Планы действий'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_Что нужно дозапросить'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +498,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Лист 10 хранит вопросы, которые нужно дозапросить для следующего шага.</t>
+          <t>Лист 09 хранит вопросы, которые нужно дозапросить для следующего шага.</t>
         </is>
       </c>
     </row>
@@ -510,99 +508,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Plan ID</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Связанный Barrier ID</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Связанное ожидание клиента</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Тип действия</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Описание действия</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Ответственная роль</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Срок или период</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Как проверить выполнение без ожидания следующего опроса</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Ожидаемый эффект</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K1"/>
-  <dataValidations count="2">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Устранение,Сдерживание,Профилактика,Эскалация,Коммуникационное действие,Обучение,Контроль,Изменение процесса,Пересмотр KPI,Другое"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Сделать,В работе,Сделано,Неизвестно"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -663,19 +568,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="39" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -686,66 +593,76 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>External project ID</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Рабочий код проекта</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>Направление проекта</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Масштаб проекта</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Операционная модель</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Известные регионы</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Основная операционная модель</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Дополнительные операционные контуры</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Этап жизненного цикла</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Статус проекта</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Дата старта</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Краткое описание проекта</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозаполнить</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:L1"/>
   <dataValidations count="5">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"FMCG,Электроника,КАФ,Промо,Обучение,Аудит,Смешанное,Другое"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Локальный,Региональный,Федеральный,Межрегиональный,Неизвестно"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Мерчендайзинг,Совмещенный мерчендайзинг,Промо / консультирование,КАФ / кадровое администрирование,Обучение,Аудит / контроль качества,Аналитика / отчетность,Смешанная,Другое"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Запуск,Стабилизация,Развитие,Удержание,Перезапуск,Риск,Закрытие,Неизвестно"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Активный,Завершен,Пилот,Под риском,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
@@ -759,18 +676,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,47 +697,42 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Роль ЛПР</t>
+          <t>External LPR ID</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>Роль / зона влияния</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>Уровень влияния</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Участвовал в блиц-опросах</t>
-        </is>
-      </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Участвовал в операционных опросах</t>
+          <t>Статус активности</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Периоды, где встречается ЛПР</t>
+          <t>Предполагаемое отношение к OPEN/услуге</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Предполагаемое отношение к OPEN/услуге</t>
+          <t>Основание вывода</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Основание вывода</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
+          <t>Комментарий для ручного уточнения</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -836,13 +747,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -853,44 +764,44 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>External LPR ID</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Важность</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Критичность</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Источник</t>
-        </is>
-      </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Доказательство из комментария</t>
+          <t>Источник вывода</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Период</t>
+          <t>Доказательство / короткая цитата</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Период / источник</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Уверенность вывода</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
@@ -904,108 +815,129 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
     <col width="31" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Survey ID</t>
+          <t>Barrier ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Project ID</t>
+          <t>Название барьера</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Тип опроса</t>
+          <t>Тип барьера</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Год</t>
+          <t>Временной статус</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Период / дата</t>
+          <t>Описание барьера</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>LPR ID</t>
+          <t>Критичность</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Вопрос</t>
+          <t>Связанный LPR ID</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Оценка</t>
+          <t>External LPR ID</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Комментарий клиента</t>
+          <t>Связанная важность ЛПР</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Тема комментария</t>
+          <t>Связанный KPI</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Тональность</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>Критичность</t>
+          <t>Доказательство / короткая цитата</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>Комментарий полезен для CJM</t>
+          <t>Период первого появления</t>
         </is>
       </c>
       <c r="N1" s="2" t="inlineStr">
         <is>
-          <t>Почему полезен / не полезен</t>
+          <t>Период последнего появления</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Статус барьера</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Статус актуальности</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Уверенность вывода</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:Q1"/>
+  <dataValidations count="4">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Блиц,Операционный"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Позитивная,Нейтральная,Негативная,Смешанная,Неизвестно"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Коммуникация,Качество исполнения,Отчетность,Сроки,Персонал,KPI,Стоимость,Обучение,Контроль,Ожидания,Организация процесса,Другое"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Было,Есть сейчас,Может возникнуть,Повторяется"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Открыт,В работе,Сдержан,Решен,Мониторинг,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1018,60 +950,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="33" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="31" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Barrier ID</t>
+          <t>Expectation ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Название барьера</t>
+          <t>Ожидание клиента</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Тип барьера</t>
+          <t>Тип ожидания</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Временной статус</t>
+          <t>Явное или неявное</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Описание барьера</t>
+          <t>Критичность</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Критичность</t>
+          <t>Связанный LPR ID</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Связанный LPR ID</t>
+          <t>External LPR ID</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
@@ -1091,44 +1021,31 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Доказательство из комментария</t>
+          <t>Доказательство / короткая цитата</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>Период первого появления</t>
+          <t>Статус актуальности</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>Период последнего появления</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
+          <t>Уверенность вывода</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
-  <dataValidations count="4">
+  <autoFilter ref="A1:M1"/>
+  <dataValidations count="3">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Коммуникация,Качество исполнения,Отчетность,Сроки,Персонал,KPI,Стоимость,Обучение,Контроль,Ожидания,Организация процесса,Другое"</formula1>
+      <formula1>"Скорость,Качество,Отчетность,Инициативность,Прозрачность,Стоимость,Экспертиза,Предсказуемость,Минимум ручного контроля,Гибкость,Соблюдение договоренностей,Другое"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Было,Есть сейчас,Может возникнуть,Повторяется"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Явное,Неявное,Неизвестно"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Открыт,В работе,Сдержан,Решен,Мониторинг,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1141,95 +1058,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="33" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Expectation ID</t>
+          <t>KPI ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Ожидание клиента</t>
+          <t>Название KPI / критерия успеха</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Тип ожидания</t>
+          <t>Тип KPI</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Явное или неявное</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Критичность</t>
+          <t>Статус актуальности</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Связанный LPR ID</t>
+          <t>Связанное ожидание клиента</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Связанная важность ЛПР</t>
+          <t>Связанный барьер</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Связанный KPI</t>
+          <t>Критичность для клиента</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Источник</t>
+          <t>Комментарий</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Доказательство из комментария</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Как можно проверить выполнение без ожидания следующего годового опроса</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
+          <t>Требует подтверждения</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
-  <dataValidations count="3">
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Скорость,Качество,Отчетность,Инициативность,Прозрачность,Стоимость,Экспертиза,Предсказуемость,Минимум ручного контроля,Гибкость,Соблюдение договоренностей,Другое"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Явное,Неявное,Неизвестно"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+  <autoFilter ref="A1:J1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1243,89 +1142,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="41" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>KPI ID</t>
+          <t>Communication ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Название KPI / критерия успеха</t>
+          <t>Сторона клиента: LPR ID или роль</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Тип KPI</t>
+          <t>External LPR ID</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Это KPI из тендера или текущий KPI</t>
+          <t>Сторона OPEN: роль</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Критичность для клиента</t>
+          <t>Тема взаимодействия</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Связанное ожидание клиента</t>
+          <t>Канал</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Связанный барьер</t>
+          <t>Частота</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Источник данных</t>
+          <t>Критичность</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Что считается нормой</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Что считается тревогой</t>
+          <t>Статус актуальности</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Что считается критическим отклонением</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Что нужно дозапросить</t>
+          <t>Комментарий</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+  <autoFilter ref="A1:K1"/>
+  <dataValidations count="3">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Встреча,Звонок,Почта,Мессенджер,Отчет,BI-дашборд,Другое,Неизвестно"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"По запросу,Еженедельно,Раз в две недели,Ежемесячно,Ежеквартально,Редко,Неизвестно"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
       <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1339,84 +1238,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Communication ID</t>
+          <t>Plan ID</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Сторона клиента</t>
+          <t>Связанный Barrier ID</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Сторона OPEN</t>
+          <t>Связанное Expectation ID</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Тема взаимодействия</t>
+          <t>Тип действия</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Канал</t>
+          <t>Описание действия</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Частота</t>
+          <t>Ответственная роль</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Критичность</t>
+          <t>Срок / период</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Есть риск разрыва коммуникации</t>
+          <t>Статус</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Основание вывода</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Что нужно дозапросить</t>
+          <t>Статус подтверждения</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Ожидаемый эффект</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Встреча,Звонок,Почта,Мессенджер,Отчет,BI-дашборд,Другое,Неизвестно"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"По запросу,Еженедельно,Раз в две недели,Ежемесячно,Ежеквартально,Редко,Неизвестно"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
-      <formula1>"Высокая,Средняя,Низкая,Неизвестно"</formula1>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Устранение,Сдерживание,Профилактика,Эскалация,Коммуникационное действие,Обучение,Контроль,Изменение процесса,Пересмотр KPI,Другое"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Сделать,В работе,Сделано,Неизвестно"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Выберите значение из MVP-справочника." prompt="Можно выбрать значение из списка." type="list">
+      <formula1>"Подтвержденный план,Черновик,AI-гипотеза,Требует согласования"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>